<commit_message>
Actualizar Planillas COF Web con soporte Anexo 4 y mejoras
</commit_message>
<xml_diff>
--- a/backend/plantilla/INFO.xlsx
+++ b/backend/plantilla/INFO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Desktop\Aplicaciones Metropol\planillas-cof-web\backend\plantilla\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB92BDDD-5053-4F0B-B6D4-E5CCAF7AFFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4CE5E0-53D2-4CA9-A4D8-E614838031C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3AA81BD4-89D4-4836-A3C3-AA400A713FDB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="78">
   <si>
     <t>unidad</t>
   </si>
@@ -56,9 +56,6 @@
     <t>AlfaU9</t>
   </si>
   <si>
-    <t>OmegaU8</t>
-  </si>
-  <si>
     <t>Condell</t>
   </si>
   <si>
@@ -270,6 +267,12 @@
   </si>
   <si>
     <t>CODIGO TS SERVICIO</t>
+  </si>
+  <si>
+    <t>AlfaU8</t>
+  </si>
+  <si>
+    <t>OmegaU9</t>
   </si>
 </sst>
 </file>
@@ -691,7 +694,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -702,10 +705,10 @@
         <v>120</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
       </c>
       <c r="E2" s="4">
         <v>812</v>
@@ -719,10 +722,10 @@
         <v>410</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3" s="4">
         <v>841</v>
@@ -733,16 +736,16 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
       <c r="E4" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -750,10 +753,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E5" s="4">
         <v>801</v>
@@ -764,10 +767,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6" s="4">
         <v>817</v>
@@ -778,10 +781,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E7" s="4">
         <v>824</v>
@@ -792,10 +795,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E8" s="4">
         <v>828</v>
@@ -806,13 +809,13 @@
         <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="E9" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -823,7 +826,7 @@
         <v>105</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E10" s="4">
         <v>805</v>
@@ -834,10 +837,10 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E11" s="4">
         <v>803</v>
@@ -848,10 +851,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E12" s="4">
         <v>809</v>
@@ -859,13 +862,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E13" s="4">
         <v>820</v>
@@ -873,13 +876,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E14" s="4">
         <v>829</v>
@@ -887,27 +890,27 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B16" s="2">
         <v>722</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E16" s="4">
         <v>822</v>
@@ -915,13 +918,13 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E17" s="4">
         <v>807</v>
@@ -929,13 +932,13 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E18" s="4">
         <v>808</v>
@@ -943,13 +946,13 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E19" s="4">
         <v>810</v>
@@ -957,13 +960,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E20" s="4">
         <v>813</v>
@@ -971,13 +974,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E21" s="4">
         <v>816</v>
@@ -985,13 +988,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E22" s="4">
         <v>818</v>
@@ -999,27 +1002,27 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E24" s="4">
         <v>825</v>
@@ -1027,13 +1030,13 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E25" s="4">
         <v>826</v>
@@ -1041,13 +1044,13 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E26" s="4">
         <v>832</v>
@@ -1055,13 +1058,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E27" s="4">
         <v>836</v>
@@ -1069,13 +1072,13 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E28" s="4">
         <v>837</v>
@@ -1083,27 +1086,27 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E30" s="4">
         <v>902</v>
@@ -1111,27 +1114,27 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E32" s="4">
         <v>904</v>
@@ -1139,13 +1142,13 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E33" s="4">
         <v>919</v>
@@ -1153,13 +1156,13 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E34" s="4">
         <v>933</v>
@@ -1167,13 +1170,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E35" s="4">
         <v>918</v>
@@ -1181,13 +1184,13 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B36" s="2">
         <v>124</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E36" s="4">
         <v>964</v>
@@ -1195,41 +1198,41 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E39" s="4">
         <v>932</v>
@@ -1237,27 +1240,27 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E41" s="4">
         <v>935</v>
@@ -1265,13 +1268,13 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E42" s="4">
         <v>938</v>
@@ -1279,13 +1282,13 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E43" s="4">
         <v>945</v>
@@ -1293,41 +1296,41 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E46" s="4">
         <v>953</v>
@@ -1335,13 +1338,13 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B47" s="2">
         <v>102</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E47" s="4">
         <v>962</v>
@@ -1349,13 +1352,13 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B48" s="2">
         <v>712</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E48" s="4">
         <v>967</v>
@@ -1363,13 +1366,13 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E49" s="4">
         <v>922</v>
@@ -1377,27 +1380,27 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E51" s="4">
         <v>925</v>
@@ -1405,13 +1408,13 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E52" s="4">
         <v>926</v>
@@ -1419,13 +1422,13 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E53" s="4">
         <v>929</v>
@@ -1433,13 +1436,13 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E54" s="4">
         <v>940</v>
@@ -1447,16 +1450,16 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>4</v>
+        <v>76</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>